<commit_message>
solicitudes aclaradas y pulidas
</commit_message>
<xml_diff>
--- a/docs/plantillas/RRH-FOR-VAR-001_Comprobante_Aumento_de_sueldo.xlsx
+++ b/docs/plantillas/RRH-FOR-VAR-001_Comprobante_Aumento_de_sueldo.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comprobante" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Comprobante'!$A$1:$AD$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Comprobante'!$A$1:$AD$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,22 +545,22 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>29</col>
       <colOff>0</colOff>
-      <row>35</row>
+      <row>38</row>
       <rowOff>0</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -575,22 +575,22 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>39</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <to>
       <col>29</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>43</row>
       <rowOff>0</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -928,19 +928,19 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>6</col>
       <colOff>0</colOff>
-      <row>36</row>
-      <rowOff>143827</rowOff>
+      <row>33</row>
+      <rowOff>125730</rowOff>
     </from>
-    <ext cx="209550" cy="209550"/>
+    <ext cx="247650" cy="247650"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -953,9 +953,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>13</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>39</row>
       <rowOff>143827</rowOff>
     </from>
     <ext cx="209550" cy="209550"/>
@@ -978,9 +978,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>15</col>
+      <col>13</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>39</row>
       <rowOff>143827</rowOff>
     </from>
     <ext cx="209550" cy="209550"/>
@@ -1003,9 +1003,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>15</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>39</row>
       <rowOff>143827</rowOff>
     </from>
     <ext cx="209550" cy="209550"/>
@@ -1028,9 +1028,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>24</col>
+      <col>22</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>39</row>
       <rowOff>143827</rowOff>
     </from>
     <ext cx="209550" cy="209550"/>
@@ -1041,6 +1041,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>143827</rowOff>
+    </from>
+    <ext cx="209550" cy="209550"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1294,7 +1319,7 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>21945</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="285750" cy="298322"/>
@@ -1341,11 +1366,11 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>69348</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5143500" cy="201368"/>
-    <xdr:sp macro="" textlink="$B$35">
+    <xdr:sp macro="" textlink="$B$38">
       <xdr:nvSpPr>
         <xdr:cNvPr id="9007" name="Seccion3"/>
         <xdr:cNvSpPr txBox="1"/>
@@ -1821,7 +1846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD42"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.285714285714286" customWidth="1" min="1" max="1"/>
@@ -2901,7 +2926,7 @@
       <c r="I31" s="10" t="n"/>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>Motivo</t>
+          <t>Fecha efectiva</t>
         </is>
       </c>
       <c r="K31" s="8" t="n"/>
@@ -2925,7 +2950,7 @@
       <c r="AC31" s="1" t="n"/>
       <c r="AD31" s="1" t="n"/>
     </row>
-    <row r="32" ht="51" customHeight="1">
+    <row r="32" ht="24" customHeight="1">
       <c r="A32" s="1" t="n"/>
       <c r="B32" s="1" t="n"/>
       <c r="C32" s="7" t="n"/>
@@ -2957,229 +2982,207 @@
       <c r="AC32" s="1" t="n"/>
       <c r="AD32" s="1" t="n"/>
     </row>
-    <row r="33" ht="7.5" customHeight="1">
+    <row r="33" ht="6.75" customHeight="1">
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="1" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
-      <c r="I33" s="16" t="n"/>
-      <c r="J33" s="16" t="n"/>
-      <c r="K33" s="16" t="n"/>
-      <c r="L33" s="16" t="n"/>
-      <c r="M33" s="16" t="n"/>
-      <c r="N33" s="16" t="n"/>
-      <c r="O33" s="16" t="n"/>
-      <c r="P33" s="16" t="n"/>
-      <c r="Q33" s="16" t="n"/>
-      <c r="R33" s="16" t="n"/>
-      <c r="S33" s="16" t="n"/>
-      <c r="T33" s="16" t="n"/>
-      <c r="U33" s="16" t="n"/>
-      <c r="V33" s="16" t="n"/>
-      <c r="W33" s="16" t="n"/>
-      <c r="X33" s="16" t="n"/>
-      <c r="Y33" s="16" t="n"/>
-      <c r="Z33" s="16" t="n"/>
-      <c r="AA33" s="16" t="n"/>
-      <c r="AB33" s="17" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
+      <c r="K33" s="8" t="n"/>
+      <c r="L33" s="8" t="n"/>
+      <c r="M33" s="8" t="n"/>
+      <c r="N33" s="8" t="n"/>
+      <c r="O33" s="8" t="n"/>
+      <c r="P33" s="8" t="n"/>
+      <c r="Q33" s="8" t="n"/>
+      <c r="R33" s="8" t="n"/>
+      <c r="S33" s="8" t="n"/>
+      <c r="T33" s="8" t="n"/>
+      <c r="U33" s="8" t="n"/>
+      <c r="V33" s="8" t="n"/>
+      <c r="W33" s="8" t="n"/>
+      <c r="X33" s="8" t="n"/>
+      <c r="Y33" s="8" t="n"/>
+      <c r="Z33" s="8" t="n"/>
+      <c r="AA33" s="8" t="n"/>
+      <c r="AB33" s="13" t="n"/>
       <c r="AC33" s="1" t="n"/>
       <c r="AD33" s="1" t="n"/>
     </row>
-    <row r="34" ht="13.5" customHeight="1">
+    <row r="34" ht="15" customHeight="1">
       <c r="A34" s="1" t="n"/>
       <c r="B34" s="1" t="n"/>
-      <c r="C34" s="1" t="n"/>
-      <c r="D34" s="1" t="n"/>
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="1" t="n"/>
-      <c r="H34" s="1" t="n"/>
-      <c r="I34" s="1" t="n"/>
-      <c r="J34" s="1" t="n"/>
-      <c r="K34" s="1" t="n"/>
-      <c r="L34" s="1" t="n"/>
-      <c r="M34" s="1" t="n"/>
-      <c r="N34" s="1" t="n"/>
-      <c r="O34" s="1" t="n"/>
-      <c r="P34" s="1" t="n"/>
-      <c r="Q34" s="1" t="n"/>
-      <c r="R34" s="1" t="n"/>
-      <c r="S34" s="1" t="n"/>
-      <c r="T34" s="1" t="n"/>
-      <c r="U34" s="1" t="n"/>
-      <c r="V34" s="1" t="n"/>
-      <c r="W34" s="1" t="n"/>
-      <c r="X34" s="1" t="n"/>
-      <c r="Y34" s="1" t="n"/>
-      <c r="Z34" s="1" t="n"/>
-      <c r="AA34" s="1" t="n"/>
-      <c r="AB34" s="1" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="10" t="n"/>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>Motivo</t>
+        </is>
+      </c>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="8" t="n"/>
+      <c r="M34" s="8" t="n"/>
+      <c r="N34" s="8" t="n"/>
+      <c r="O34" s="8" t="n"/>
+      <c r="P34" s="8" t="n"/>
+      <c r="Q34" s="8" t="n"/>
+      <c r="R34" s="8" t="n"/>
+      <c r="S34" s="8" t="n"/>
+      <c r="T34" s="8" t="n"/>
+      <c r="U34" s="8" t="n"/>
+      <c r="V34" s="8" t="n"/>
+      <c r="W34" s="8" t="n"/>
+      <c r="X34" s="8" t="n"/>
+      <c r="Y34" s="8" t="n"/>
+      <c r="Z34" s="8" t="n"/>
+      <c r="AA34" s="8" t="n"/>
+      <c r="AB34" s="13" t="n"/>
       <c r="AC34" s="1" t="n"/>
       <c r="AD34" s="1" t="n"/>
     </row>
-    <row r="35" ht="27" customHeight="1">
+    <row r="35" ht="51" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="10" t="n"/>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="8" t="n"/>
+      <c r="L35" s="8" t="n"/>
+      <c r="M35" s="8" t="n"/>
+      <c r="N35" s="8" t="n"/>
+      <c r="O35" s="8" t="n"/>
+      <c r="P35" s="8" t="n"/>
+      <c r="Q35" s="8" t="n"/>
+      <c r="R35" s="8" t="n"/>
+      <c r="S35" s="8" t="n"/>
+      <c r="T35" s="8" t="n"/>
+      <c r="U35" s="8" t="n"/>
+      <c r="V35" s="8" t="n"/>
+      <c r="W35" s="8" t="n"/>
+      <c r="X35" s="8" t="n"/>
+      <c r="Y35" s="8" t="n"/>
+      <c r="Z35" s="8" t="n"/>
+      <c r="AA35" s="8" t="n"/>
+      <c r="AB35" s="13" t="n"/>
+      <c r="AC35" s="1" t="n"/>
+      <c r="AD35" s="1" t="n"/>
+    </row>
+    <row r="36" ht="7.5" customHeight="1">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="16" t="n"/>
+      <c r="H36" s="16" t="n"/>
+      <c r="I36" s="16" t="n"/>
+      <c r="J36" s="16" t="n"/>
+      <c r="K36" s="16" t="n"/>
+      <c r="L36" s="16" t="n"/>
+      <c r="M36" s="16" t="n"/>
+      <c r="N36" s="16" t="n"/>
+      <c r="O36" s="16" t="n"/>
+      <c r="P36" s="16" t="n"/>
+      <c r="Q36" s="16" t="n"/>
+      <c r="R36" s="16" t="n"/>
+      <c r="S36" s="16" t="n"/>
+      <c r="T36" s="16" t="n"/>
+      <c r="U36" s="16" t="n"/>
+      <c r="V36" s="16" t="n"/>
+      <c r="W36" s="16" t="n"/>
+      <c r="X36" s="16" t="n"/>
+      <c r="Y36" s="16" t="n"/>
+      <c r="Z36" s="16" t="n"/>
+      <c r="AA36" s="16" t="n"/>
+      <c r="AB36" s="17" t="n"/>
+      <c r="AC36" s="1" t="n"/>
+      <c r="AD36" s="1" t="n"/>
+    </row>
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
+      <c r="K37" s="1" t="n"/>
+      <c r="L37" s="1" t="n"/>
+      <c r="M37" s="1" t="n"/>
+      <c r="N37" s="1" t="n"/>
+      <c r="O37" s="1" t="n"/>
+      <c r="P37" s="1" t="n"/>
+      <c r="Q37" s="1" t="n"/>
+      <c r="R37" s="1" t="n"/>
+      <c r="S37" s="1" t="n"/>
+      <c r="T37" s="1" t="n"/>
+      <c r="U37" s="1" t="n"/>
+      <c r="V37" s="1" t="n"/>
+      <c r="W37" s="1" t="n"/>
+      <c r="X37" s="1" t="n"/>
+      <c r="Y37" s="1" t="n"/>
+      <c r="Z37" s="1" t="n"/>
+      <c r="AA37" s="1" t="n"/>
+      <c r="AB37" s="1" t="n"/>
+      <c r="AC37" s="1" t="n"/>
+      <c r="AD37" s="1" t="n"/>
+    </row>
+    <row r="38" ht="27" customHeight="1">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>APROBACIONES</t>
         </is>
       </c>
-      <c r="C35" s="1" t="n"/>
-      <c r="D35" s="1" t="n"/>
-      <c r="E35" s="1" t="n"/>
-      <c r="F35" s="1" t="n"/>
-      <c r="G35" s="1" t="n"/>
-      <c r="H35" s="1" t="n"/>
-      <c r="I35" s="1" t="n"/>
-      <c r="J35" s="1" t="n"/>
-      <c r="K35" s="1" t="n"/>
-      <c r="L35" s="1" t="n"/>
-      <c r="M35" s="1" t="n"/>
-      <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
-      <c r="P35" s="1" t="n"/>
-      <c r="Q35" s="1" t="n"/>
-      <c r="R35" s="1" t="n"/>
-      <c r="S35" s="1" t="n"/>
-      <c r="T35" s="1" t="n"/>
-      <c r="U35" s="1" t="n"/>
-      <c r="V35" s="1" t="n"/>
-      <c r="W35" s="1" t="n"/>
-      <c r="X35" s="1" t="n"/>
-      <c r="Y35" s="1" t="n"/>
-      <c r="Z35" s="1" t="n"/>
-      <c r="AA35" s="1" t="n"/>
-      <c r="AB35" s="1" t="n"/>
-      <c r="AC35" s="1" t="n"/>
-      <c r="AD35" s="1" t="n"/>
-    </row>
-    <row r="36" ht="9.75" customHeight="1">
-      <c r="A36" s="1" t="n"/>
-      <c r="B36" s="1" t="n"/>
-      <c r="C36" s="1" t="n"/>
-      <c r="D36" s="1" t="n"/>
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-      <c r="G36" s="1" t="n"/>
-      <c r="H36" s="1" t="n"/>
-      <c r="I36" s="1" t="n"/>
-      <c r="J36" s="1" t="n"/>
-      <c r="K36" s="1" t="n"/>
-      <c r="L36" s="1" t="n"/>
-      <c r="M36" s="1" t="n"/>
-      <c r="N36" s="1" t="n"/>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
-      <c r="Q36" s="1" t="n"/>
-      <c r="R36" s="1" t="n"/>
-      <c r="S36" s="1" t="n"/>
-      <c r="T36" s="1" t="n"/>
-      <c r="U36" s="1" t="n"/>
-      <c r="V36" s="1" t="n"/>
-      <c r="W36" s="1" t="n"/>
-      <c r="X36" s="1" t="n"/>
-      <c r="Y36" s="1" t="n"/>
-      <c r="Z36" s="1" t="n"/>
-      <c r="AA36" s="1" t="n"/>
-      <c r="AB36" s="1" t="n"/>
-      <c r="AC36" s="1" t="n"/>
-      <c r="AD36" s="1" t="n"/>
-    </row>
-    <row r="37" ht="39" customHeight="1">
-      <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="18" t="inlineStr">
-        <is>
-          <t>N°</t>
-        </is>
-      </c>
-      <c r="E37" s="19" t="n"/>
-      <c r="F37" s="19" t="n"/>
-      <c r="G37" s="19" t="n"/>
-      <c r="H37" s="20" t="inlineStr">
-        <is>
-          <t>Aprobador</t>
-        </is>
-      </c>
-      <c r="I37" s="21" t="n"/>
-      <c r="J37" s="21" t="n"/>
-      <c r="K37" s="21" t="n"/>
-      <c r="L37" s="21" t="n"/>
-      <c r="M37" s="22" t="inlineStr">
-        <is>
-          <t>Decisión</t>
-        </is>
-      </c>
-      <c r="N37" s="23" t="n"/>
-      <c r="O37" s="24" t="inlineStr">
-        <is>
-          <t>Asignado</t>
-        </is>
-      </c>
-      <c r="P37" s="25" t="n"/>
-      <c r="Q37" s="25" t="n"/>
-      <c r="R37" s="25" t="n"/>
-      <c r="S37" s="25" t="n"/>
-      <c r="T37" s="25" t="n"/>
-      <c r="U37" s="25" t="n"/>
-      <c r="V37" s="26" t="inlineStr">
-        <is>
-          <t>Decidido</t>
-        </is>
-      </c>
-      <c r="W37" s="27" t="n"/>
-      <c r="X37" s="28" t="inlineStr">
-        <is>
-          <t>Tiempo de respuesta</t>
-        </is>
-      </c>
-      <c r="Y37" s="29" t="n"/>
-      <c r="Z37" s="29" t="n"/>
-      <c r="AA37" s="29" t="n"/>
-      <c r="AB37" s="1" t="n"/>
-      <c r="AC37" s="1" t="n"/>
-      <c r="AD37" s="1" t="n"/>
-    </row>
-    <row r="38" ht="39.75" customHeight="1">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="n"/>
       <c r="C38" s="1" t="n"/>
-      <c r="D38" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="31" t="n"/>
-      <c r="F38" s="31" t="n"/>
-      <c r="G38" s="31" t="n"/>
-      <c r="H38" s="32" t="n"/>
-      <c r="I38" s="31" t="n"/>
-      <c r="J38" s="31" t="n"/>
-      <c r="K38" s="31" t="n"/>
-      <c r="L38" s="31" t="n"/>
-      <c r="M38" s="33" t="n"/>
-      <c r="N38" s="31" t="n"/>
-      <c r="O38" s="34" t="n"/>
-      <c r="P38" s="31" t="n"/>
-      <c r="Q38" s="31" t="n"/>
-      <c r="R38" s="31" t="n"/>
-      <c r="S38" s="31" t="n"/>
-      <c r="T38" s="31" t="n"/>
-      <c r="U38" s="31" t="n"/>
-      <c r="V38" s="34" t="n"/>
-      <c r="W38" s="31" t="n"/>
-      <c r="X38" s="35" t="n"/>
-      <c r="Y38" s="31" t="n"/>
-      <c r="Z38" s="31" t="n"/>
-      <c r="AA38" s="31" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
+      <c r="K38" s="1" t="n"/>
+      <c r="L38" s="1" t="n"/>
+      <c r="M38" s="1" t="n"/>
+      <c r="N38" s="1" t="n"/>
+      <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="n"/>
+      <c r="Q38" s="1" t="n"/>
+      <c r="R38" s="1" t="n"/>
+      <c r="S38" s="1" t="n"/>
+      <c r="T38" s="1" t="n"/>
+      <c r="U38" s="1" t="n"/>
+      <c r="V38" s="1" t="n"/>
+      <c r="W38" s="1" t="n"/>
+      <c r="X38" s="1" t="n"/>
+      <c r="Y38" s="1" t="n"/>
+      <c r="Z38" s="1" t="n"/>
+      <c r="AA38" s="1" t="n"/>
       <c r="AB38" s="1" t="n"/>
       <c r="AC38" s="1" t="n"/>
       <c r="AD38" s="1" t="n"/>
     </row>
-    <row r="39" ht="13.5" customHeight="1">
+    <row r="39" ht="9.75" customHeight="1">
       <c r="A39" s="1" t="n"/>
       <c r="B39" s="1" t="n"/>
       <c r="C39" s="1" t="n"/>
@@ -3211,43 +3214,165 @@
       <c r="AC39" s="1" t="n"/>
       <c r="AD39" s="1" t="n"/>
     </row>
-    <row r="40" ht="5.25" customHeight="1">
+    <row r="40" ht="39" customHeight="1">
       <c r="A40" s="1" t="n"/>
       <c r="B40" s="1" t="n"/>
       <c r="C40" s="1" t="n"/>
-      <c r="D40" s="1" t="n"/>
-      <c r="E40" s="1" t="n"/>
-      <c r="F40" s="1" t="n"/>
-      <c r="G40" s="1" t="n"/>
-      <c r="H40" s="1" t="n"/>
-      <c r="I40" s="1" t="n"/>
-      <c r="J40" s="1" t="n"/>
-      <c r="K40" s="1" t="n"/>
-      <c r="L40" s="1" t="n"/>
-      <c r="M40" s="1" t="n"/>
-      <c r="N40" s="1" t="n"/>
-      <c r="O40" s="1" t="n"/>
-      <c r="P40" s="1" t="n"/>
-      <c r="Q40" s="1" t="n"/>
-      <c r="R40" s="1" t="n"/>
-      <c r="S40" s="1" t="n"/>
-      <c r="T40" s="1" t="n"/>
-      <c r="U40" s="1" t="n"/>
-      <c r="V40" s="1" t="n"/>
-      <c r="W40" s="1" t="n"/>
-      <c r="X40" s="1" t="n"/>
-      <c r="Y40" s="1" t="n"/>
-      <c r="Z40" s="1" t="n"/>
-      <c r="AA40" s="1" t="n"/>
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="20" t="inlineStr">
+        <is>
+          <t>Aprobador</t>
+        </is>
+      </c>
+      <c r="I40" s="21" t="n"/>
+      <c r="J40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
+      <c r="M40" s="22" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="N40" s="23" t="n"/>
+      <c r="O40" s="24" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="P40" s="25" t="n"/>
+      <c r="Q40" s="25" t="n"/>
+      <c r="R40" s="25" t="n"/>
+      <c r="S40" s="25" t="n"/>
+      <c r="T40" s="25" t="n"/>
+      <c r="U40" s="25" t="n"/>
+      <c r="V40" s="26" t="inlineStr">
+        <is>
+          <t>Decidido</t>
+        </is>
+      </c>
+      <c r="W40" s="27" t="n"/>
+      <c r="X40" s="28" t="inlineStr">
+        <is>
+          <t>Tiempo de respuesta</t>
+        </is>
+      </c>
+      <c r="Y40" s="29" t="n"/>
+      <c r="Z40" s="29" t="n"/>
+      <c r="AA40" s="29" t="n"/>
       <c r="AB40" s="1" t="n"/>
       <c r="AC40" s="1" t="n"/>
       <c r="AD40" s="1" t="n"/>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="39.75" customHeight="1">
       <c r="A41" s="1" t="n"/>
       <c r="B41" s="1" t="n"/>
       <c r="C41" s="1" t="n"/>
-      <c r="D41" s="36" t="inlineStr">
+      <c r="D41" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="31" t="n"/>
+      <c r="G41" s="31" t="n"/>
+      <c r="H41" s="32" t="n"/>
+      <c r="I41" s="31" t="n"/>
+      <c r="J41" s="31" t="n"/>
+      <c r="K41" s="31" t="n"/>
+      <c r="L41" s="31" t="n"/>
+      <c r="M41" s="33" t="n"/>
+      <c r="N41" s="31" t="n"/>
+      <c r="O41" s="34" t="n"/>
+      <c r="P41" s="31" t="n"/>
+      <c r="Q41" s="31" t="n"/>
+      <c r="R41" s="31" t="n"/>
+      <c r="S41" s="31" t="n"/>
+      <c r="T41" s="31" t="n"/>
+      <c r="U41" s="31" t="n"/>
+      <c r="V41" s="34" t="n"/>
+      <c r="W41" s="31" t="n"/>
+      <c r="X41" s="35" t="n"/>
+      <c r="Y41" s="31" t="n"/>
+      <c r="Z41" s="31" t="n"/>
+      <c r="AA41" s="31" t="n"/>
+      <c r="AB41" s="1" t="n"/>
+      <c r="AC41" s="1" t="n"/>
+      <c r="AD41" s="1" t="n"/>
+    </row>
+    <row r="42" ht="13.5" customHeight="1">
+      <c r="A42" s="1" t="n"/>
+      <c r="B42" s="1" t="n"/>
+      <c r="C42" s="1" t="n"/>
+      <c r="D42" s="1" t="n"/>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="n"/>
+      <c r="G42" s="1" t="n"/>
+      <c r="H42" s="1" t="n"/>
+      <c r="I42" s="1" t="n"/>
+      <c r="J42" s="1" t="n"/>
+      <c r="K42" s="1" t="n"/>
+      <c r="L42" s="1" t="n"/>
+      <c r="M42" s="1" t="n"/>
+      <c r="N42" s="1" t="n"/>
+      <c r="O42" s="1" t="n"/>
+      <c r="P42" s="1" t="n"/>
+      <c r="Q42" s="1" t="n"/>
+      <c r="R42" s="1" t="n"/>
+      <c r="S42" s="1" t="n"/>
+      <c r="T42" s="1" t="n"/>
+      <c r="U42" s="1" t="n"/>
+      <c r="V42" s="1" t="n"/>
+      <c r="W42" s="1" t="n"/>
+      <c r="X42" s="1" t="n"/>
+      <c r="Y42" s="1" t="n"/>
+      <c r="Z42" s="1" t="n"/>
+      <c r="AA42" s="1" t="n"/>
+      <c r="AB42" s="1" t="n"/>
+      <c r="AC42" s="1" t="n"/>
+      <c r="AD42" s="1" t="n"/>
+    </row>
+    <row r="43" ht="5.25" customHeight="1">
+      <c r="A43" s="1" t="n"/>
+      <c r="B43" s="1" t="n"/>
+      <c r="C43" s="1" t="n"/>
+      <c r="D43" s="1" t="n"/>
+      <c r="E43" s="1" t="n"/>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="n"/>
+      <c r="H43" s="1" t="n"/>
+      <c r="I43" s="1" t="n"/>
+      <c r="J43" s="1" t="n"/>
+      <c r="K43" s="1" t="n"/>
+      <c r="L43" s="1" t="n"/>
+      <c r="M43" s="1" t="n"/>
+      <c r="N43" s="1" t="n"/>
+      <c r="O43" s="1" t="n"/>
+      <c r="P43" s="1" t="n"/>
+      <c r="Q43" s="1" t="n"/>
+      <c r="R43" s="1" t="n"/>
+      <c r="S43" s="1" t="n"/>
+      <c r="T43" s="1" t="n"/>
+      <c r="U43" s="1" t="n"/>
+      <c r="V43" s="1" t="n"/>
+      <c r="W43" s="1" t="n"/>
+      <c r="X43" s="1" t="n"/>
+      <c r="Y43" s="1" t="n"/>
+      <c r="Z43" s="1" t="n"/>
+      <c r="AA43" s="1" t="n"/>
+      <c r="AB43" s="1" t="n"/>
+      <c r="AC43" s="1" t="n"/>
+      <c r="AD43" s="1" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="1" t="n"/>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3292,118 +3417,121 @@
           </r>
         </is>
       </c>
-      <c r="E41" s="1" t="n"/>
-      <c r="F41" s="1" t="n"/>
-      <c r="G41" s="1" t="n"/>
-      <c r="H41" s="1" t="n"/>
-      <c r="I41" s="1" t="n"/>
-      <c r="J41" s="1" t="n"/>
-      <c r="K41" s="1" t="n"/>
-      <c r="L41" s="1" t="n"/>
-      <c r="M41" s="1" t="n"/>
-      <c r="N41" s="1" t="n"/>
-      <c r="O41" s="1" t="n"/>
-      <c r="P41" s="1" t="n"/>
-      <c r="Q41" s="1" t="n"/>
-      <c r="R41" s="1" t="n"/>
-      <c r="S41" s="1" t="n"/>
-      <c r="T41" s="1" t="n"/>
-      <c r="U41" s="1" t="n"/>
-      <c r="V41" s="1" t="n"/>
-      <c r="W41" s="1" t="n"/>
-      <c r="X41" s="1" t="n"/>
-      <c r="Y41" s="1" t="n"/>
-      <c r="Z41" s="1" t="n"/>
-      <c r="AA41" s="1" t="n"/>
-      <c r="AB41" s="1" t="n"/>
-      <c r="AC41" s="1" t="n"/>
-      <c r="AD41" s="1" t="n"/>
-    </row>
-    <row r="42" ht="9" customHeight="1">
-      <c r="A42" s="1" t="n"/>
-      <c r="B42" s="1" t="n"/>
-      <c r="C42" s="1" t="n"/>
-      <c r="D42" s="1" t="n"/>
-      <c r="E42" s="1" t="n"/>
-      <c r="F42" s="1" t="n"/>
-      <c r="G42" s="1" t="n"/>
-      <c r="H42" s="1" t="n"/>
-      <c r="I42" s="1" t="n"/>
-      <c r="J42" s="1" t="n"/>
-      <c r="K42" s="1" t="n"/>
-      <c r="L42" s="1" t="n"/>
-      <c r="M42" s="1" t="n"/>
-      <c r="N42" s="1" t="n"/>
-      <c r="O42" s="1" t="n"/>
-      <c r="P42" s="1" t="n"/>
-      <c r="Q42" s="1" t="n"/>
-      <c r="R42" s="1" t="n"/>
-      <c r="S42" s="1" t="n"/>
-      <c r="T42" s="1" t="n"/>
-      <c r="U42" s="1" t="n"/>
-      <c r="V42" s="1" t="n"/>
-      <c r="W42" s="1" t="n"/>
-      <c r="X42" s="1" t="n"/>
-      <c r="Y42" s="1" t="n"/>
-      <c r="Z42" s="1" t="n"/>
-      <c r="AA42" s="1" t="n"/>
-      <c r="AB42" s="1" t="n"/>
-      <c r="AC42" s="1" t="n"/>
-      <c r="AD42" s="1" t="n"/>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
+      <c r="K44" s="1" t="n"/>
+      <c r="L44" s="1" t="n"/>
+      <c r="M44" s="1" t="n"/>
+      <c r="N44" s="1" t="n"/>
+      <c r="O44" s="1" t="n"/>
+      <c r="P44" s="1" t="n"/>
+      <c r="Q44" s="1" t="n"/>
+      <c r="R44" s="1" t="n"/>
+      <c r="S44" s="1" t="n"/>
+      <c r="T44" s="1" t="n"/>
+      <c r="U44" s="1" t="n"/>
+      <c r="V44" s="1" t="n"/>
+      <c r="W44" s="1" t="n"/>
+      <c r="X44" s="1" t="n"/>
+      <c r="Y44" s="1" t="n"/>
+      <c r="Z44" s="1" t="n"/>
+      <c r="AA44" s="1" t="n"/>
+      <c r="AB44" s="1" t="n"/>
+      <c r="AC44" s="1" t="n"/>
+      <c r="AD44" s="1" t="n"/>
+    </row>
+    <row r="45" ht="9" customHeight="1">
+      <c r="A45" s="1" t="n"/>
+      <c r="B45" s="1" t="n"/>
+      <c r="C45" s="1" t="n"/>
+      <c r="D45" s="1" t="n"/>
+      <c r="E45" s="1" t="n"/>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="n"/>
+      <c r="H45" s="1" t="n"/>
+      <c r="I45" s="1" t="n"/>
+      <c r="J45" s="1" t="n"/>
+      <c r="K45" s="1" t="n"/>
+      <c r="L45" s="1" t="n"/>
+      <c r="M45" s="1" t="n"/>
+      <c r="N45" s="1" t="n"/>
+      <c r="O45" s="1" t="n"/>
+      <c r="P45" s="1" t="n"/>
+      <c r="Q45" s="1" t="n"/>
+      <c r="R45" s="1" t="n"/>
+      <c r="S45" s="1" t="n"/>
+      <c r="T45" s="1" t="n"/>
+      <c r="U45" s="1" t="n"/>
+      <c r="V45" s="1" t="n"/>
+      <c r="W45" s="1" t="n"/>
+      <c r="X45" s="1" t="n"/>
+      <c r="Y45" s="1" t="n"/>
+      <c r="Z45" s="1" t="n"/>
+      <c r="AA45" s="1" t="n"/>
+      <c r="AB45" s="1" t="n"/>
+      <c r="AC45" s="1" t="n"/>
+      <c r="AD45" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="54">
+    <mergeCell ref="J31:P31"/>
     <mergeCell ref="U16:Z16"/>
+    <mergeCell ref="X41:AA41"/>
     <mergeCell ref="S9:T10"/>
     <mergeCell ref="S28:T29"/>
     <mergeCell ref="U25:Z25"/>
     <mergeCell ref="F25:I26"/>
-    <mergeCell ref="H38:L38"/>
     <mergeCell ref="S15:T16"/>
     <mergeCell ref="F12:I13"/>
-    <mergeCell ref="V38:W38"/>
     <mergeCell ref="J12:P12"/>
+    <mergeCell ref="H41:L41"/>
     <mergeCell ref="U13:Z13"/>
-    <mergeCell ref="D38:G38"/>
-    <mergeCell ref="O38:U38"/>
+    <mergeCell ref="F34:I35"/>
+    <mergeCell ref="H40:L40"/>
     <mergeCell ref="J18:P18"/>
     <mergeCell ref="U12:Z12"/>
     <mergeCell ref="F18:I19"/>
-    <mergeCell ref="X38:AA38"/>
-    <mergeCell ref="O37:U37"/>
     <mergeCell ref="U28:Z28"/>
+    <mergeCell ref="J34:Z34"/>
     <mergeCell ref="U18:Z18"/>
+    <mergeCell ref="X40:AA40"/>
     <mergeCell ref="J29:P29"/>
+    <mergeCell ref="V40:W40"/>
     <mergeCell ref="J10:P10"/>
     <mergeCell ref="J28:P28"/>
     <mergeCell ref="F31:I32"/>
+    <mergeCell ref="M40:N40"/>
     <mergeCell ref="J19:P19"/>
     <mergeCell ref="U29:Z29"/>
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="J13:P13"/>
     <mergeCell ref="S12:T13"/>
     <mergeCell ref="U10:Z10"/>
     <mergeCell ref="F9:I10"/>
     <mergeCell ref="S25:T26"/>
-    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="J35:Z35"/>
     <mergeCell ref="J9:P9"/>
     <mergeCell ref="U19:Z19"/>
     <mergeCell ref="U26:Z26"/>
     <mergeCell ref="F28:I29"/>
     <mergeCell ref="J15:P15"/>
-    <mergeCell ref="H37:L37"/>
-    <mergeCell ref="J32:Z32"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="V41:W41"/>
     <mergeCell ref="U9:Z9"/>
     <mergeCell ref="S18:T19"/>
-    <mergeCell ref="D37:G37"/>
-    <mergeCell ref="X37:AA37"/>
-    <mergeCell ref="J31:Z31"/>
+    <mergeCell ref="D41:G41"/>
+    <mergeCell ref="O41:U41"/>
     <mergeCell ref="U15:Z15"/>
-    <mergeCell ref="M38:N38"/>
     <mergeCell ref="J26:P26"/>
-    <mergeCell ref="V37:W37"/>
     <mergeCell ref="J16:P16"/>
+    <mergeCell ref="J32:P32"/>
     <mergeCell ref="F15:I16"/>
     <mergeCell ref="J25:P25"/>
+    <mergeCell ref="O40:U40"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.45" header="0.5" footer="0.5"/>

</xml_diff>